<commit_message>
Treat merged title and banner cells as one cell in header detection
Exporters write a merged cell's value into every cell it covers, so a
banner such as "Card XXXX (EUR)" spanning the table looked like a row of
labels: it was taken as the header and the real header above it was
rejected. Header detection now counts distinct values per row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/files/imports/bank_formats.xlsx
+++ b/test/fixtures/files/imports/bank_formats.xlsx
@@ -21,7 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary_block" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spanish" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unknown_amount_header" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes_only" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="merged_banners" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes_only" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -857,6 +858,151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Encours prélevé : Fin août 2026</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Encours prélevé : Fin août 2026</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Encours prélevé : Fin août 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R.I.B. : 10278 02619 00099999901 - 08/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>R.I.B. : 10278 02619 00099999901 - 08/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>R.I.B. : 10278 02619 00099999901 - 08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Liste de vos comptes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Liste de vos comptes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Liste de vos comptes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Libellé</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Montant</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Carte Mastercard XXXXXXXXXXXX9999 (EUR)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Carte Mastercard XXXXXXXXXXXX9999 (EUR)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Carte Mastercard XXXXXXXXXXXX9999 (EUR)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Carte Mastercard XXXXXXXXXXXX9999 (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OPENAI CHATGPT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>-23</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ENTERPRISE RENT</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>200</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Translate the Excel import into every supported locale
The import screens were only translated into English and French. Move
its strings to config/locales/views/xlsx_imports/<locale>.yml and add
all 18 supported locales, with a test that each locale has every key
and that the sheet selection page renders in each of them.

Header detection now also recognises label, amount, debit/credit,
balance and value-date headers in those languages (Polish, Russian,
Ukrainian, Turkish, Hungarian, Vietnamese, Chinese, Catalan, Norwegian,
Romanian, Portuguese...), covered by new fixture sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/files/imports/bank_formats.xlsx
+++ b/test/fixtures/files/imports/bank_formats.xlsx
@@ -22,7 +22,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spanish" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unknown_amount_header" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="merged_banners" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes_only" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="polish" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="russian" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="turkish" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chinese" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes_only" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1003,21 +1007,303 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Ce fichier a été généré automatiquement.</t>
+          <t>Historia rachunku</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Data operacji</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Opis</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Obciążenia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Uznania</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Saldo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Biedronka</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>-45.2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>45356</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Wynagrodzenie</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5200</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6155</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Выписка по счёту</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aucune opération sur la période.</t>
-        </is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Сумма</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Остаток</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Пятёрочка</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>-1250.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8749.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45384</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Зарплата</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>68749.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Hesap hareketleri</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>İşlem tarihi</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Açıklama</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Tutar</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bakiye</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45414</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Market alışverişi</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>-320.75</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4679.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>45415</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Maaş</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>29679.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易明细</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>交易日期</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>摘要</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>支出</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>收入</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>余额</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45444</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>超市购物</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>911.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45445</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>工资</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>8911.5</v>
       </c>
     </row>
   </sheetData>
@@ -1103,6 +1389,34 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Ce fichier a été généré automatiquement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aucune opération sur la période.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>